<commit_message>
Updated risk sheet 22/02
</commit_message>
<xml_diff>
--- a/Plan/CW Risks.xlsx
+++ b/Plan/CW Risks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stuartbaker/Desktop/University/Year2/Software Engineering/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stuartbaker/Documents/GitHub/Software-Engineering-Project/Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86162115-A730-1F4C-A956-525F745F17A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7137E90-030E-B741-A075-E59D5ABC3982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15980" xr2:uid="{96C42A70-5923-F145-81DA-CC33F505D3E0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>Affects</t>
   </si>
@@ -168,6 +168,36 @@
   </si>
   <si>
     <t>Weekly team meetings and daily communication to track progress; allow slack time between tasks</t>
+  </si>
+  <si>
+    <t>Illness</t>
+  </si>
+  <si>
+    <t>Share workload of the unwell member; flexibility in deadlines and meetings</t>
+  </si>
+  <si>
+    <t>Poor communication (medium); luck (high); cold weather (high)</t>
+  </si>
+  <si>
+    <t>Communincate when unwell and its affect on performance; change meetings and wokrload to accommodate</t>
+  </si>
+  <si>
+    <t>Traffic, trains and buses</t>
+  </si>
+  <si>
+    <t>Missing uni, meetings; unable to work; Fall behind</t>
+  </si>
+  <si>
+    <t>Plan ahead by checking disruptions before leaving; communicate with team</t>
+  </si>
+  <si>
+    <t>Poor travel planning (high); misfortune (medium)</t>
+  </si>
+  <si>
+    <t>Inform of any disruptions to team; alert team when you will be late/ miss events</t>
+  </si>
+  <si>
+    <t>Missing uni; missing meetings; lowers morale; lateness</t>
   </si>
 </sst>
 </file>
@@ -596,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FF717A5-D0E1-0E43-BC29-58ACCCC5A807}">
-  <dimension ref="B2:F10"/>
+  <dimension ref="B2:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="6" width="40.83203125" customWidth="1"/>
@@ -755,6 +785,40 @@
         <v>43</v>
       </c>
     </row>
+    <row r="11" spans="2:6" ht="60" x14ac:dyDescent="0.2">
+      <c r="B11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="40" x14ac:dyDescent="0.2">
+      <c r="B12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>